<commit_message>
Redesign database.xlsx parsing and project-scoped folder matching rules
- Column 2: part number, column 3: model, project columns: per-project designators
- Traverse workspace -> project folders -> chip test subfolders
- Match bracket-wrapped folder names by designator, model, or mixed variants
- Matching is scoped to the current project column in database.xlsx

Co-authored-by: Jiahui-a <Jiahui-a@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/cascon-database-sync/templates/database_template.xlsx
+++ b/cascon-database-sync/templates/database_template.xlsx
@@ -413,74 +413,110 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>序号</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>料号</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
           <t>型号</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>位号</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>料号</t>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>ProjectA</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>ProjectB</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>C12345-001</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
           <t>STM32F103C8T6</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>U1</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>C12345-001</t>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>U5</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>C12345-002</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
           <t>GD32F303CCT6</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>U2</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>C12345-002</t>
-        </is>
-      </c>
+      <c r="E3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>C12345-003</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
           <t>W25Q128JVSIQ</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>U3</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>C12345-003</t>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>U8</t>
         </is>
       </c>
     </row>

</xml_diff>